<commit_message>
Cambiadas algunas fórmulas de la excel para ajustarse a lo dado en clase...
</commit_message>
<xml_diff>
--- a/data/xlsx/resultados-fase-1.xlsx
+++ b/data/xlsx/resultados-fase-1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\menda\Desktop\Diego\Universidad\Tercero\AC\teamwork-ac-2025\data\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E3A1960-66C5-44E5-90C9-136C245B82D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EFAAAAC-27E2-4D9D-A4A9-9EE6C0C72C7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{64E32888-7FF9-4962-B0B2-27FE6E737F4E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Prueba 1</t>
   </si>
@@ -77,10 +77,16 @@
     <t>Desviación Típica</t>
   </si>
   <si>
-    <t>Extr. Inf. Interv. Conf</t>
-  </si>
-  <si>
-    <t>Extr. Sup. Interv. Conf.</t>
+    <t>Extr. Inf. Interv. Conf (t Student)</t>
+  </si>
+  <si>
+    <t>Extr. Sup. Interv. Conf. (t Student)</t>
+  </si>
+  <si>
+    <t>Extr. Sup. Interv. Conf. (TCL)</t>
+  </si>
+  <si>
+    <t>Extr. Inf. Interv. Conf. (TCL)</t>
   </si>
 </sst>
 </file>
@@ -473,15 +479,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C88A2E26-47F6-4350-B42D-F2D297B06200}">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:Q4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="2" max="10" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.88671875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.5546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="27.21875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="23.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -525,8 +536,14 @@
       <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
+      <c r="P1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -565,7 +582,7 @@
         <v>9.6399999999999988</v>
       </c>
       <c r="M2" s="3">
-        <f>_xlfn.STDEV.S(B2:K2)</f>
+        <f>STDEVA(B2:K2)</f>
         <v>0.1685229954635272</v>
       </c>
       <c r="N2" s="3">
@@ -576,8 +593,16 @@
         <f>L2 + _xlfn.CONFIDENCE.T(0.05,M2,10)/2</f>
         <v>9.7002770443098481</v>
       </c>
+      <c r="P2" s="3">
+        <f xml:space="preserve"> L2 - 2*M2</f>
+        <v>9.3029540090729448</v>
+      </c>
+      <c r="Q2" s="3">
+        <f xml:space="preserve"> L2 + 2*M2</f>
+        <v>9.9770459909270528</v>
+      </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -594,7 +619,7 @@
       <c r="N3" s="3"/>
       <c r="O3" s="3"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>

</xml_diff>

<commit_message>
Cambiados los resultados de la excel tras las modificaiones del algoritmo
</commit_message>
<xml_diff>
--- a/data/xlsx/resultados-fase-1.xlsx
+++ b/data/xlsx/resultados-fase-1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\menda\Desktop\Diego\Universidad\Tercero\AC\teamwork-ac-2025\data\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EFAAAAC-27E2-4D9D-A4A9-9EE6C0C72C7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83606DF8-E37C-400C-B970-25269C9A3DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{64E32888-7FF9-4962-B0B2-27FE6E737F4E}"/>
   </bookViews>
@@ -548,58 +548,58 @@
         <v>10</v>
       </c>
       <c r="B2" s="3">
-        <v>9.68</v>
+        <v>10.86</v>
       </c>
       <c r="C2" s="3">
-        <v>9.74</v>
+        <v>10.59</v>
       </c>
       <c r="D2" s="3">
-        <v>9.17</v>
+        <v>10.27</v>
       </c>
       <c r="E2" s="3">
-        <v>9.6199999999999992</v>
+        <v>10.32</v>
       </c>
       <c r="F2" s="3">
-        <v>9.69</v>
+        <v>10.86</v>
       </c>
       <c r="G2" s="3">
-        <v>9.68</v>
+        <v>10.67</v>
       </c>
       <c r="H2" s="3">
-        <v>9.68</v>
+        <v>10.71</v>
       </c>
       <c r="I2" s="3">
-        <v>9.7200000000000006</v>
+        <v>10.91</v>
       </c>
       <c r="J2" s="3">
-        <v>9.73</v>
+        <v>10.42</v>
       </c>
       <c r="K2" s="3">
-        <v>9.69</v>
+        <v>10.51</v>
       </c>
       <c r="L2" s="3">
         <f>AVERAGE(B2:K2)</f>
-        <v>9.6399999999999988</v>
+        <v>10.612</v>
       </c>
       <c r="M2" s="3">
         <f>STDEVA(B2:K2)</f>
-        <v>0.1685229954635272</v>
+        <v>0.22967610043518047</v>
       </c>
       <c r="N2" s="3">
         <f>L2 - _xlfn.CONFIDENCE.T(0.05,M2,10)/2</f>
-        <v>9.5797229556901495</v>
+        <v>10.529849807708642</v>
       </c>
       <c r="O2" s="3">
         <f>L2 + _xlfn.CONFIDENCE.T(0.05,M2,10)/2</f>
-        <v>9.7002770443098481</v>
+        <v>10.694150192291358</v>
       </c>
       <c r="P2" s="3">
         <f xml:space="preserve"> L2 - 2*M2</f>
-        <v>9.3029540090729448</v>
+        <v>10.152647799129639</v>
       </c>
       <c r="Q2" s="3">
         <f xml:space="preserve"> L2 + 2*M2</f>
-        <v>9.9770459909270528</v>
+        <v>11.071352200870361</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">

</xml_diff>